<commit_message>
Source Data: final tables for manuscript revision 3
Replaces the earlier sync (#2). source_data/ now mirrors the manuscript repository
at its revision-3 state: ED Fig 3c regenerated from the released probabilities;
Fig 5g / ED Fig 7a,d aligned to the plotted bars and error bars; Fig 5f reduced to
the panel's four values; GPT-5.2-vision rows dropped from Fig 6b-d; ED Fig 7b,e,i
given their own sheets; Fig 7d extended with the non-selected candidates and the
round-0 origin; Supp Fig 3c CIs as drawn; every system label as printed on its panel
(TLAgent -> TissueLab etc.), with full names kept in system_description.
Workbooks rebuilt (14 workbooks, 57 sheets).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/workbooks/Source_Data_ED_Fig2.xlsx
+++ b/source_data/workbooks/Source_Data_ED_Fig2.xlsx
@@ -85,28 +85,28 @@
     <t>MedGemma</t>
   </si>
   <si>
+    <t>M3D</t>
+  </si>
+  <si>
+    <t>GPT-4o-vision</t>
+  </si>
+  <si>
+    <t>GPT-5-vision</t>
+  </si>
+  <si>
+    <t>GPT-5.4-vision</t>
+  </si>
+  <si>
+    <t>GPT-4o-agent</t>
+  </si>
+  <si>
     <t>MAM</t>
   </si>
   <si>
-    <t>M3D</t>
-  </si>
-  <si>
-    <t>GPT-4o-vision</t>
-  </si>
-  <si>
-    <t>GPT-5-vision</t>
-  </si>
-  <si>
-    <t>GPT-5.4-vision</t>
-  </si>
-  <si>
-    <t>GPT-4o-agent</t>
-  </si>
-  <si>
     <t>MedAgent-Pro</t>
   </si>
   <si>
-    <t>TLAgent</t>
+    <t>TissueLab</t>
   </si>
   <si>
     <t>accuracy</t>
@@ -121,21 +121,21 @@
     <t>0.4533</t>
   </si>
   <si>
+    <t>no evaluable output</t>
+  </si>
+  <si>
+    <t>0.5733</t>
+  </si>
+  <si>
+    <t>0.5307</t>
+  </si>
+  <si>
+    <t>0.48</t>
+  </si>
+  <si>
     <t>0.5413</t>
   </si>
   <si>
-    <t>no evaluable output</t>
-  </si>
-  <si>
-    <t>0.5733</t>
-  </si>
-  <si>
-    <t>0.5307</t>
-  </si>
-  <si>
-    <t>0.48</t>
-  </si>
-  <si>
     <t>0.464</t>
   </si>
   <si>
@@ -157,18 +157,18 @@
     <t>-0.1377</t>
   </si>
   <si>
+    <t>0.1867</t>
+  </si>
+  <si>
+    <t>0.1081</t>
+  </si>
+  <si>
+    <t>0.0643</t>
+  </si>
+  <si>
     <t>0.0829</t>
   </si>
   <si>
-    <t>0.1867</t>
-  </si>
-  <si>
-    <t>0.1081</t>
-  </si>
-  <si>
-    <t>0.0643</t>
-  </si>
-  <si>
     <t>-0.0628</t>
   </si>
   <si>
@@ -184,16 +184,16 @@
     <t>0.7333</t>
   </si>
   <si>
+    <t>0.896</t>
+  </si>
+  <si>
+    <t>0.928</t>
+  </si>
+  <si>
+    <t>0.368</t>
+  </si>
+  <si>
     <t>0.0667</t>
-  </si>
-  <si>
-    <t>0.896</t>
-  </si>
-  <si>
-    <t>0.928</t>
-  </si>
-  <si>
-    <t>0.368</t>
   </si>
   <si>
     <t>0.0747</t>
@@ -762,28 +762,13 @@
         <v>75</v>
       </c>
       <c r="J4">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="K4">
         <v>5</v>
       </c>
       <c r="L4" t="s">
         <v>34</v>
-      </c>
-      <c r="M4">
-        <v>0.0335</v>
-      </c>
-      <c r="N4">
-        <v>0.4507</v>
-      </c>
-      <c r="O4">
-        <v>0.6347</v>
-      </c>
-      <c r="P4">
-        <v>0.4507</v>
-      </c>
-      <c r="Q4">
-        <v>0.6347</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -815,7 +800,7 @@
         <v>75</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="K5">
         <v>5</v>
@@ -823,6 +808,21 @@
       <c r="L5" t="s">
         <v>35</v>
       </c>
+      <c r="M5">
+        <v>0.0094</v>
+      </c>
+      <c r="N5">
+        <v>0.4613</v>
+      </c>
+      <c r="O5">
+        <v>0.6853</v>
+      </c>
+      <c r="P5">
+        <v>0.4613</v>
+      </c>
+      <c r="Q5">
+        <v>0.6853</v>
+      </c>
     </row>
     <row r="6" spans="1:17">
       <c r="A6">
@@ -853,28 +853,13 @@
         <v>75</v>
       </c>
       <c r="J6">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="K6">
         <v>5</v>
       </c>
       <c r="L6" t="s">
-        <v>36</v>
-      </c>
-      <c r="M6">
-        <v>0.0094</v>
-      </c>
-      <c r="N6">
-        <v>0.4613</v>
-      </c>
-      <c r="O6">
-        <v>0.6853</v>
-      </c>
-      <c r="P6">
-        <v>0.4613</v>
-      </c>
-      <c r="Q6">
-        <v>0.6853</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -906,13 +891,28 @@
         <v>75</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="K7">
         <v>5</v>
       </c>
       <c r="L7" t="s">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="M7">
+        <v>0.006</v>
+      </c>
+      <c r="N7">
+        <v>0.4187</v>
+      </c>
+      <c r="O7">
+        <v>0.64</v>
+      </c>
+      <c r="P7">
+        <v>0.4187</v>
+      </c>
+      <c r="Q7">
+        <v>0.64</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -944,7 +944,7 @@
         <v>75</v>
       </c>
       <c r="J8">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="K8">
         <v>5</v>
@@ -953,19 +953,19 @@
         <v>37</v>
       </c>
       <c r="M8">
-        <v>0.006</v>
+        <v>0.0365</v>
       </c>
       <c r="N8">
-        <v>0.4187</v>
+        <v>0.3893</v>
       </c>
       <c r="O8">
-        <v>0.64</v>
+        <v>0.5707</v>
       </c>
       <c r="P8">
-        <v>0.4187</v>
+        <v>0.3893</v>
       </c>
       <c r="Q8">
-        <v>0.64</v>
+        <v>0.5707</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -997,7 +997,7 @@
         <v>75</v>
       </c>
       <c r="J9">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="K9">
         <v>5</v>
@@ -1006,19 +1006,19 @@
         <v>38</v>
       </c>
       <c r="M9">
-        <v>0.0365</v>
+        <v>0.0335</v>
       </c>
       <c r="N9">
-        <v>0.3893</v>
+        <v>0.4507</v>
       </c>
       <c r="O9">
-        <v>0.5707</v>
+        <v>0.6347</v>
       </c>
       <c r="P9">
-        <v>0.3893</v>
+        <v>0.4507</v>
       </c>
       <c r="Q9">
-        <v>0.5707</v>
+        <v>0.6347</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -1341,28 +1341,13 @@
         <v>75</v>
       </c>
       <c r="J4">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="K4">
         <v>5</v>
       </c>
       <c r="L4" t="s">
-        <v>46</v>
-      </c>
-      <c r="M4">
-        <v>0.0852</v>
-      </c>
-      <c r="N4">
-        <v>-0.0541</v>
-      </c>
-      <c r="O4">
-        <v>0.2167</v>
-      </c>
-      <c r="P4">
-        <v>-0.0541</v>
-      </c>
-      <c r="Q4">
-        <v>0.2167</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -1394,13 +1379,28 @@
         <v>75</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="K5">
         <v>5</v>
       </c>
       <c r="L5" t="s">
-        <v>35</v>
+        <v>46</v>
+      </c>
+      <c r="M5">
+        <v>0.0246</v>
+      </c>
+      <c r="N5">
+        <v>-0.0348</v>
+      </c>
+      <c r="O5">
+        <v>0.3741</v>
+      </c>
+      <c r="P5">
+        <v>-0.0348</v>
+      </c>
+      <c r="Q5">
+        <v>0.3741</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -1432,28 +1432,13 @@
         <v>75</v>
       </c>
       <c r="J6">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="K6">
         <v>5</v>
       </c>
       <c r="L6" t="s">
-        <v>47</v>
-      </c>
-      <c r="M6">
-        <v>0.0246</v>
-      </c>
-      <c r="N6">
-        <v>-0.0348</v>
-      </c>
-      <c r="O6">
-        <v>0.3741</v>
-      </c>
-      <c r="P6">
-        <v>-0.0348</v>
-      </c>
-      <c r="Q6">
-        <v>0.3741</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -1485,13 +1470,28 @@
         <v>75</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="K7">
         <v>5</v>
       </c>
       <c r="L7" t="s">
-        <v>35</v>
+        <v>47</v>
+      </c>
+      <c r="M7">
+        <v>0.0541</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0.1859</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>0.1859</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -1523,7 +1523,7 @@
         <v>75</v>
       </c>
       <c r="J8">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="K8">
         <v>5</v>
@@ -1532,19 +1532,19 @@
         <v>48</v>
       </c>
       <c r="M8">
-        <v>0.0541</v>
+        <v>0.0936</v>
       </c>
       <c r="N8">
-        <v>0</v>
+        <v>-0.0529</v>
       </c>
       <c r="O8">
-        <v>0.1859</v>
+        <v>0.1752</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>-0.0529</v>
       </c>
       <c r="Q8">
-        <v>0.1859</v>
+        <v>0.1752</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -1576,7 +1576,7 @@
         <v>75</v>
       </c>
       <c r="J9">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="K9">
         <v>5</v>
@@ -1585,19 +1585,19 @@
         <v>49</v>
       </c>
       <c r="M9">
-        <v>0.0936</v>
+        <v>0.0852</v>
       </c>
       <c r="N9">
-        <v>-0.0529</v>
+        <v>-0.0541</v>
       </c>
       <c r="O9">
-        <v>0.1752</v>
+        <v>0.2167</v>
       </c>
       <c r="P9">
-        <v>-0.0529</v>
+        <v>-0.0541</v>
       </c>
       <c r="Q9">
-        <v>0.1752</v>
+        <v>0.2167</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -1920,28 +1920,13 @@
         <v>75</v>
       </c>
       <c r="J4">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="K4">
         <v>5</v>
       </c>
       <c r="L4" t="s">
-        <v>55</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4">
-        <v>0.0133</v>
-      </c>
-      <c r="O4">
-        <v>0.1333</v>
-      </c>
-      <c r="P4">
-        <v>0.0133</v>
-      </c>
-      <c r="Q4">
-        <v>0.1333</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -1973,13 +1958,28 @@
         <v>75</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="K5">
         <v>5</v>
       </c>
       <c r="L5" t="s">
-        <v>35</v>
+        <v>55</v>
+      </c>
+      <c r="M5">
+        <v>0.0112</v>
+      </c>
+      <c r="N5">
+        <v>0.8267</v>
+      </c>
+      <c r="O5">
+        <v>0.9573</v>
+      </c>
+      <c r="P5">
+        <v>0.8267</v>
+      </c>
+      <c r="Q5">
+        <v>0.9573</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -2011,28 +2011,13 @@
         <v>75</v>
       </c>
       <c r="J6">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="K6">
         <v>5</v>
       </c>
       <c r="L6" t="s">
-        <v>56</v>
-      </c>
-      <c r="M6">
-        <v>0.0112</v>
-      </c>
-      <c r="N6">
-        <v>0.8267</v>
-      </c>
-      <c r="O6">
-        <v>0.9573</v>
-      </c>
-      <c r="P6">
-        <v>0.8267</v>
-      </c>
-      <c r="Q6">
-        <v>0.9573</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -2064,13 +2049,28 @@
         <v>75</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="K7">
         <v>5</v>
       </c>
       <c r="L7" t="s">
-        <v>35</v>
+        <v>56</v>
+      </c>
+      <c r="M7">
+        <v>0.0152</v>
+      </c>
+      <c r="N7">
+        <v>0.8693</v>
+      </c>
+      <c r="O7">
+        <v>0.976</v>
+      </c>
+      <c r="P7">
+        <v>0.8693</v>
+      </c>
+      <c r="Q7">
+        <v>0.976</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -2102,7 +2102,7 @@
         <v>75</v>
       </c>
       <c r="J8">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="K8">
         <v>5</v>
@@ -2111,19 +2111,19 @@
         <v>57</v>
       </c>
       <c r="M8">
-        <v>0.0152</v>
+        <v>0.1339</v>
       </c>
       <c r="N8">
-        <v>0.8693</v>
+        <v>0.32</v>
       </c>
       <c r="O8">
-        <v>0.976</v>
+        <v>0.4187</v>
       </c>
       <c r="P8">
-        <v>0.8693</v>
+        <v>0.32</v>
       </c>
       <c r="Q8">
-        <v>0.976</v>
+        <v>0.4187</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -2155,7 +2155,7 @@
         <v>75</v>
       </c>
       <c r="J9">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="K9">
         <v>5</v>
@@ -2164,19 +2164,19 @@
         <v>58</v>
       </c>
       <c r="M9">
-        <v>0.1339</v>
+        <v>0</v>
       </c>
       <c r="N9">
-        <v>0.32</v>
+        <v>0.0133</v>
       </c>
       <c r="O9">
-        <v>0.4187</v>
+        <v>0.1333</v>
       </c>
       <c r="P9">
-        <v>0.32</v>
+        <v>0.0133</v>
       </c>
       <c r="Q9">
-        <v>0.4187</v>
+        <v>0.1333</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -2499,28 +2499,13 @@
         <v>75</v>
       </c>
       <c r="J4">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="K4">
         <v>5</v>
       </c>
       <c r="L4" t="s">
-        <v>44</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4">
-        <v>0</v>
-      </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
-      <c r="P4">
-        <v>0</v>
-      </c>
-      <c r="Q4">
-        <v>0</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -2552,13 +2537,28 @@
         <v>75</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="K5">
         <v>5</v>
       </c>
       <c r="L5" t="s">
-        <v>35</v>
+        <v>64</v>
+      </c>
+      <c r="M5">
+        <v>0.0081</v>
+      </c>
+      <c r="N5">
+        <v>-0.08989999999999999</v>
+      </c>
+      <c r="O5">
+        <v>-0.0121</v>
+      </c>
+      <c r="P5">
+        <v>-0.08989999999999999</v>
+      </c>
+      <c r="Q5">
+        <v>-0.0121</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -2590,28 +2590,13 @@
         <v>75</v>
       </c>
       <c r="J6">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="K6">
         <v>5</v>
       </c>
       <c r="L6" t="s">
-        <v>64</v>
-      </c>
-      <c r="M6">
-        <v>0.0081</v>
-      </c>
-      <c r="N6">
-        <v>-0.08989999999999999</v>
-      </c>
-      <c r="O6">
-        <v>-0.0121</v>
-      </c>
-      <c r="P6">
-        <v>-0.08989999999999999</v>
-      </c>
-      <c r="Q6">
-        <v>-0.0121</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -2643,13 +2628,28 @@
         <v>75</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="K7">
         <v>5</v>
       </c>
       <c r="L7" t="s">
-        <v>35</v>
+        <v>65</v>
+      </c>
+      <c r="M7">
+        <v>0.2185</v>
+      </c>
+      <c r="N7">
+        <v>-0.0407</v>
+      </c>
+      <c r="O7">
+        <v>0.4289</v>
+      </c>
+      <c r="P7">
+        <v>-0.0407</v>
+      </c>
+      <c r="Q7">
+        <v>0.4289</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -2681,28 +2681,28 @@
         <v>75</v>
       </c>
       <c r="J8">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="K8">
         <v>5</v>
       </c>
       <c r="L8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M8">
-        <v>0.2185</v>
+        <v>0.1062</v>
       </c>
       <c r="N8">
-        <v>-0.0407</v>
+        <v>-0.1738</v>
       </c>
       <c r="O8">
-        <v>0.4289</v>
+        <v>-0.0018</v>
       </c>
       <c r="P8">
-        <v>-0.0407</v>
+        <v>-0.1738</v>
       </c>
       <c r="Q8">
-        <v>0.4289</v>
+        <v>-0.0018</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -2734,28 +2734,28 @@
         <v>75</v>
       </c>
       <c r="J9">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="K9">
         <v>5</v>
       </c>
       <c r="L9" t="s">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="M9">
-        <v>0.1062</v>
+        <v>0</v>
       </c>
       <c r="N9">
-        <v>-0.1738</v>
+        <v>0</v>
       </c>
       <c r="O9">
-        <v>-0.0018</v>
+        <v>0</v>
       </c>
       <c r="P9">
-        <v>-0.1738</v>
+        <v>0</v>
       </c>
       <c r="Q9">
-        <v>-0.0018</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:17">

</xml_diff>